<commit_message>
add new test case
</commit_message>
<xml_diff>
--- a/test/ACTVN_TestCases - test.xlsx
+++ b/test/ACTVN_TestCases - test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vien1\Downloads\OceanTech\School\kiemThuNhung\nightwatch-git\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB756DA-C1FC-44C3-85A7-3F7FC438346C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62F9254B-CBC1-4F42-A555-62BE4B8CDF1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
   <si>
     <t>ID</t>
   </si>
@@ -136,34 +136,40 @@
     <t>Mở tab mới hoặc chuyển trang tới "file PDF chứa chương trình đào tạo ngành CNTT"</t>
   </si>
   <si>
-    <t>TC05</t>
+    <t xml:space="preserve">	Kiểm tra thấy "Điện thoại"; Kiểm tra thấy "Địa chỉ"; Kiểm tra thấy "Điện thoại"; Kiểm tra thấy "học viện"; Kiểm tra thấy "hôm nay"</t>
   </si>
   <si>
-    <t>Kiểm tra 'Khảo thí &amp; ĐBCL'</t>
+    <t>TC14</t>
   </si>
   <si>
-    <t>Đảm bảo có thông tin khảo thí</t>
+    <t>Kiểm tra truy cập mục 'Học bổng'</t>
+  </si>
+  <si>
+    <t>Xác minh nội dung học bổng hiện lên</t>
   </si>
   <si>
     <t>1. Mở trình duyệt
 2. Truy cập trang https://actvn.edu.vn
-3. Hover vào mục 'Đào tạo' trên navbar
-4. Click vào 'Khảo thí &amp; ĐBCL'</t>
+3. Hover vào mục 'Sinh viên' trên navbar
+4. Click vào 'Học bổng'</t>
   </si>
   <si>
     <t>Mở trình duyệt
 Truy cập trang https://actvn.edu.vn
-Di chuột đến "Đào tạo"
-Bấm vào "Khảo thí &amp; ĐBCL"</t>
+Di chuột đến "Sinh viên"
+Bấm vào "Học bổng"</t>
   </si>
   <si>
-    <t>Thông tin khảo thí được hiển thị</t>
+    <t>Hiển thị các học bổng hiện hành</t>
   </si>
   <si>
-    <t>Kiểm tra thấy "khảo thí"</t>
+    <t xml:space="preserve">        Kiểm tra thấy "Học bổng"</t>
   </si>
   <si>
-    <t xml:space="preserve">	Kiểm tra thấy "Điện thoại"; Kiểm tra thấy "Địa chỉ"; Kiểm tra thấy "Điện thoại"; Kiểm tra thấy "học viện"; Kiểm tra thấy "hôm nay"</t>
+    <t/>
+  </si>
+  <si>
+    <t>FAIL: Không tìm thấy phần tử để hover: "Sinh viên"</t>
   </si>
 </sst>
 </file>
@@ -237,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -246,6 +252,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -463,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K976"/>
+  <dimension ref="A1:M976"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -475,7 +484,7 @@
     <col min="9" max="11" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="72" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="72" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -510,7 +519,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="72" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="72" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -533,11 +542,11 @@
         <v>17</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:11" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" ht="72" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -564,36 +573,46 @@
       </c>
       <c r="K3" s="2"/>
     </row>
-    <row r="4" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="2" t="s">
+    <row r="4" spans="1:13" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="B4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="C4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="F4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="G4" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-    </row>
-    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="M4" s="4"/>
+    </row>
+    <row r="5" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -606,7 +625,7 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -619,7 +638,7 @@
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
     </row>
-    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -632,7 +651,7 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -645,7 +664,7 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -658,7 +677,7 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -671,7 +690,7 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -684,7 +703,7 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -697,7 +716,7 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -710,7 +729,7 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -723,7 +742,7 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -736,7 +755,7 @@
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>

</xml_diff>